<commit_message>
updated haushofer part provision list
</commit_message>
<xml_diff>
--- a/Bestuecker_Files/Rev.06/Haushofer_Beistellung_März2022.xlsx
+++ b/Bestuecker_Files/Rev.06/Haushofer_Beistellung_März2022.xlsx
@@ -1,30 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24827"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\UZ_A_ltc2311-16\Bestuecker_Files\Rev.06\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_a_ltc2311-16\Bestuecker_Files\Rev.06\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465099E6-88EC-481C-ADC7-9072014D273F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24650" windowHeight="11240"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="76">
   <si>
     <t>BUF634AIDR</t>
   </si>
@@ -249,12 +260,15 @@
   </si>
   <si>
     <t>https://wwwapps.ups.com/tracking/tracking.cgi?tracknum=1ZWA47976635939104&amp;requester=ST/trackdetails</t>
+  </si>
+  <si>
+    <t>Beigestellte Menge</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -313,7 +327,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -334,6 +348,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -398,7 +418,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -435,6 +455,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Gut" xfId="1" builtinId="26"/>
@@ -738,11 +766,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.6328125" customWidth="1"/>
@@ -750,14 +778,14 @@
     <col min="4" max="4" width="19.36328125" customWidth="1"/>
     <col min="5" max="5" width="23.54296875" customWidth="1"/>
     <col min="6" max="7" width="12.08984375" customWidth="1"/>
-    <col min="8" max="8" width="10.90625" customWidth="1"/>
-    <col min="9" max="9" width="17.7265625" customWidth="1"/>
-    <col min="11" max="11" width="19.54296875" customWidth="1"/>
-    <col min="12" max="12" width="63.6328125" customWidth="1"/>
-    <col min="13" max="13" width="68.36328125" customWidth="1"/>
+    <col min="8" max="9" width="10.90625" customWidth="1"/>
+    <col min="10" max="10" width="17.7265625" customWidth="1"/>
+    <col min="12" max="12" width="19.54296875" customWidth="1"/>
+    <col min="13" max="13" width="63.6328125" customWidth="1"/>
+    <col min="14" max="14" width="68.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="7" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="7" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>39</v>
       </c>
@@ -783,63 +811,69 @@
         <v>49</v>
       </c>
       <c r="I1" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:14" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="8">
+    <row r="2" spans="1:15" s="16" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="17">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="16">
         <f t="shared" ref="F2:F15" si="0">A2*$G$18</f>
         <v>20</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="16">
         <v>9</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="17">
         <v>125</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="15">
+        <v>25</v>
+      </c>
+      <c r="J2" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="9">
-        <f t="shared" ref="J2:J15" si="1">G2+H2-F2</f>
+      <c r="K2" s="17">
+        <f t="shared" ref="K2:K15" si="1">G2+H2-F2</f>
         <v>114</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="L2" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="M2" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="N2" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="O2" s="16" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:14" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="8">
+    <row r="3" spans="1:15" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="9">
         <v>1</v>
       </c>
       <c r="B3" s="8" t="s">
@@ -864,22 +898,25 @@
       <c r="H3" s="9">
         <v>50</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="14">
+        <v>50</v>
+      </c>
+      <c r="J3" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="J3" s="9">
+      <c r="K3" s="9">
         <f t="shared" si="1"/>
         <v>38</v>
       </c>
-      <c r="K3" s="11" t="s">
+      <c r="L3" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="L3" s="13" t="s">
+      <c r="M3" s="13" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:14" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="8">
+    <row r="4" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="9">
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
@@ -904,19 +941,22 @@
       <c r="H4" s="9">
         <v>25</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="14">
+        <v>25</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="J4" s="9">
+      <c r="K4" s="9">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K4" s="11" t="s">
+      <c r="L4" s="11" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:14" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="8">
+    <row r="5" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
@@ -941,19 +981,22 @@
       <c r="H5" s="9">
         <v>25</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="14">
+        <v>25</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="9">
+      <c r="K5" s="9">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K5" s="11" t="s">
+      <c r="L5" s="11" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:14" s="8" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="8">
+    <row r="6" spans="1:15" s="8" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="9">
         <v>8</v>
       </c>
       <c r="B6" s="8" t="s">
@@ -978,19 +1021,22 @@
       <c r="H6" s="9">
         <v>130</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I6" s="14">
+        <v>170</v>
+      </c>
+      <c r="J6" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="J6" s="9">
+      <c r="K6" s="9">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="L6" s="11" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" s="8" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="8">
+    <row r="7" spans="1:15" s="8" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="9">
         <v>8</v>
       </c>
       <c r="B7" s="8" t="s">
@@ -1015,19 +1061,22 @@
       <c r="H7" s="9">
         <v>170</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="14">
+        <v>170</v>
+      </c>
+      <c r="J7" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="J7" s="9">
+      <c r="K7" s="9">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="K7" s="11" t="s">
+      <c r="L7" s="11" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:14" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="8">
+    <row r="8" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="9">
         <v>1</v>
       </c>
       <c r="B8" t="s">
@@ -1050,19 +1099,22 @@
       <c r="H8">
         <v>25</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="14">
+        <v>25</v>
+      </c>
+      <c r="J8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="J8" s="9">
+      <c r="K8" s="9">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K8" s="11" t="s">
+      <c r="L8" s="11" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:14" s="8" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8">
+    <row r="9" spans="1:15" s="8" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="9">
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
@@ -1087,25 +1139,28 @@
       <c r="H9" s="9">
         <v>111</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="14">
+        <v>191</v>
+      </c>
+      <c r="J9" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="J9" s="9">
+      <c r="K9" s="9">
         <f t="shared" si="1"/>
         <v>31</v>
       </c>
-      <c r="K9" s="11" t="s">
+      <c r="L9" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="N9" s="13" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:14" s="8" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="8">
+    <row r="10" spans="1:15" s="8" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="9">
         <v>2</v>
       </c>
       <c r="B10" s="8" t="s">
@@ -1130,19 +1185,22 @@
       <c r="H10" s="9">
         <v>44</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I10" s="14">
+        <v>44</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="J10" s="9">
+      <c r="K10" s="9">
         <f t="shared" si="1"/>
         <v>52</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="L10" s="11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:14" s="8" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="8">
+    <row r="11" spans="1:15" s="8" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="9">
         <v>1</v>
       </c>
       <c r="B11" s="8" t="s">
@@ -1167,19 +1225,22 @@
       <c r="H11" s="9">
         <v>22</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="I11" s="14">
+        <v>22</v>
+      </c>
+      <c r="J11" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="J11" s="9">
+      <c r="K11" s="9">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="K11" s="11" t="s">
+      <c r="L11" s="11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:14" s="8" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="8">
+    <row r="12" spans="1:15" s="8" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="9">
         <v>1</v>
       </c>
       <c r="B12" s="8" t="s">
@@ -1199,16 +1260,19 @@
         <v>20</v>
       </c>
       <c r="G12" s="8">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H12" s="9"/>
-      <c r="J12" s="9">
+      <c r="I12" s="14">
+        <v>32</v>
+      </c>
+      <c r="K12" s="9">
         <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" s="8" customFormat="1" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" s="8" customFormat="1" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="9">
         <v>1</v>
       </c>
       <c r="B13" s="8" t="s">
@@ -1228,16 +1292,19 @@
         <v>20</v>
       </c>
       <c r="G13" s="8">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H13" s="9"/>
-      <c r="J13" s="9">
+      <c r="I13" s="14">
+        <v>22</v>
+      </c>
+      <c r="K13" s="9">
         <f t="shared" si="1"/>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A14" s="8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="9">
         <v>1</v>
       </c>
       <c r="B14" s="8" t="s">
@@ -1260,15 +1327,18 @@
         <v>32</v>
       </c>
       <c r="H14" s="9"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="9">
+      <c r="I14" s="14">
+        <v>22</v>
+      </c>
+      <c r="J14" s="8"/>
+      <c r="K14" s="9">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="K14" s="8"/>
-    </row>
-    <row r="15" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="8">
+      <c r="L14" s="8"/>
+    </row>
+    <row r="15" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="9">
         <v>16</v>
       </c>
       <c r="B15" t="s">
@@ -1293,21 +1363,24 @@
       <c r="H15">
         <v>500</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="14">
+        <v>500</v>
+      </c>
+      <c r="J15" t="s">
         <v>61</v>
       </c>
-      <c r="J15" s="9">
+      <c r="K15" s="9">
         <f t="shared" si="1"/>
         <v>180</v>
       </c>
-      <c r="K15" s="11" t="s">
+      <c r="L15" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
@@ -1320,10 +1393,10 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:K15">
-    <sortCondition ref="I1"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L15">
+    <sortCondition ref="J1"/>
   </sortState>
-  <conditionalFormatting sqref="J2:J15">
+  <conditionalFormatting sqref="K2:K15">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
@@ -1332,10 +1405,10 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="L2" r:id="rId1"/>
-    <hyperlink ref="L3" r:id="rId2"/>
-    <hyperlink ref="M2" r:id="rId3"/>
-    <hyperlink ref="L9" r:id="rId4"/>
+    <hyperlink ref="M2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="M3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N2" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="M9" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="96" orientation="landscape" r:id="rId5"/>

</xml_diff>